<commit_message>
DSV 新增 VAT 跟 Shipper 欄位擷取
- _dsv_extract_items()：費用明細行的正則表達式本來就有抓 "PPN IN IDR"
  這個群組 (ppn)，只是之前完全沒用上，這次補寫進 items 當作 vat。
- parse_dsv()：新增 header["shipper"]。這份帳單的 "ULTIMATE SHIPPER"/
  "ULTIMATE CONSIGNEE" 兩欄左右並排、擷取出來的文字黏在同一行、中間沒有
  可靠的分隔符號，沒辦法單純用正則表達式切開；但觀察使用者提供的兩份
  正確答案 (3 張發票/5 張發票)，每一張 ULTIMATE SHIPPER 的值都跟
  header["consignee"]（帳單最上面的受票公司）完全一樣，所以直接沿用
  已經可靠抓到的 consignee 值。

使用者這次提供的兩份正確答案 Excel 用現有程式碼測試都已經是 100% 正確
率，已經把 test_samples/DSV/sample1_ref.xlsx、sample2_ref.xlsx 換成這次
更新後的版本 (含 VAT/Shipper)，run_regression.py 全部 14 家供應商、所有
樣本仍維持 100% 正確率。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JhL7qxuxZLsZyoRKZr1of6
</commit_message>
<xml_diff>
--- a/test_samples/DSV/sample1_ref.xlsx
+++ b/test_samples/DSV/sample1_ref.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffrey.hu\Desktop\LC\供應商帳單\DSV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffrey.hu\Desktop\印尼供應商帳單\DSV____________OK\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EABCE7-74CA-486E-89AA-855AB8B344DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A570BE8-B17E-4479-AFB7-217678F20458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="819" xr2:uid="{B2E6A21A-966E-4572-9141-AA1879003F42}"/>
+    <workbookView xWindow="3120" yWindow="7920" windowWidth="28800" windowHeight="15315" tabRatio="819" xr2:uid="{B2E6A21A-966E-4572-9141-AA1879003F42}"/>
   </bookViews>
   <sheets>
     <sheet name="DWIHARTA" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="39">
   <si>
     <t>INVOICE DATE
 發票日期</t>
@@ -184,6 +184,15 @@
   </si>
   <si>
     <t>BEAU5996998</t>
+  </si>
+  <si>
+    <t>VAT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shipper
+出貨方</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -599,27 +608,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF1381F-552A-4924-9A7A-4C0080F73CE6}">
-  <dimension ref="A1:Q13"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:R13"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" customWidth="1"/>
-    <col min="3" max="3" width="29.453125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="15.75" customWidth="1"/>
+    <col min="3" max="3" width="29.5" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.90625" customWidth="1"/>
-    <col min="7" max="7" width="29.26953125" customWidth="1"/>
-    <col min="8" max="9" width="13.7265625" customWidth="1"/>
-    <col min="10" max="10" width="20.54296875" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.36328125" customWidth="1"/>
-    <col min="15" max="15" width="20.6328125" customWidth="1"/>
-    <col min="16" max="16" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.875" customWidth="1"/>
+    <col min="8" max="8" width="29.25" customWidth="1"/>
+    <col min="9" max="10" width="13.75" customWidth="1"/>
+    <col min="11" max="11" width="20.5" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.375" customWidth="1"/>
+    <col min="16" max="16" width="20.625" customWidth="1"/>
+    <col min="17" max="17" width="15.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" s="1" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -639,37 +648,43 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="R1" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46268</v>
       </c>
@@ -688,38 +703,44 @@
       <c r="F2">
         <v>3140183</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2">
+        <v>345420</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="3">
         <v>46311</v>
       </c>
-      <c r="I2" s="3">
+      <c r="J2" s="3">
         <v>46269</v>
       </c>
-      <c r="J2" t="s">
-        <v>24</v>
-      </c>
       <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
         <v>30</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>25</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>29</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>8.4710000000000001</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>27</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>28</v>
       </c>
+      <c r="R2" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46268</v>
       </c>
@@ -738,38 +759,44 @@
       <c r="F3">
         <v>546601</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3">
+        <v>60126</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="3">
+      <c r="I3" s="3">
         <v>46311</v>
       </c>
-      <c r="I3" s="3">
+      <c r="J3" s="3">
         <v>46269</v>
       </c>
-      <c r="J3" t="s">
-        <v>24</v>
-      </c>
       <c r="K3" t="s">
         <v>24</v>
       </c>
       <c r="L3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" t="s">
         <v>25</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>29</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>8.4710000000000001</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>27</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>28</v>
       </c>
+      <c r="R3" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>46268</v>
       </c>
@@ -788,38 +815,44 @@
       <c r="F4">
         <v>169309</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4">
+        <v>18624</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>46311</v>
       </c>
-      <c r="I4" s="3">
+      <c r="J4" s="3">
         <v>46269</v>
       </c>
-      <c r="J4" t="s">
-        <v>24</v>
-      </c>
       <c r="K4" t="s">
         <v>24</v>
       </c>
       <c r="L4" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" t="s">
         <v>25</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>29</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>8.4710000000000001</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>27</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>28</v>
       </c>
+      <c r="R4" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>46268</v>
       </c>
@@ -838,38 +871,44 @@
       <c r="F5">
         <v>622000</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5">
+        <v>68420</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>46311</v>
       </c>
-      <c r="I5" s="3">
+      <c r="J5" s="3">
         <v>46269</v>
       </c>
-      <c r="J5" t="s">
-        <v>24</v>
-      </c>
       <c r="K5" t="s">
         <v>24</v>
       </c>
       <c r="L5" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" t="s">
         <v>25</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>29</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>8.4710000000000001</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>27</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>28</v>
       </c>
+      <c r="R5" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>46268</v>
       </c>
@@ -888,38 +927,44 @@
       <c r="F6">
         <v>2945566</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6">
+        <v>324012</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="3">
         <v>46311</v>
       </c>
-      <c r="I6" s="3">
+      <c r="J6" s="3">
         <v>46269</v>
       </c>
-      <c r="J6" t="s">
-        <v>24</v>
-      </c>
       <c r="K6" t="s">
         <v>24</v>
       </c>
       <c r="L6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" t="s">
         <v>25</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>29</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>7.9459999999999997</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>26</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>33</v>
       </c>
+      <c r="R6" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>46268</v>
       </c>
@@ -938,38 +983,44 @@
       <c r="F7">
         <v>546601</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7">
+        <v>60126</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>46311</v>
       </c>
-      <c r="I7" s="3">
+      <c r="J7" s="3">
         <v>46269</v>
       </c>
-      <c r="J7" t="s">
-        <v>24</v>
-      </c>
       <c r="K7" t="s">
         <v>24</v>
       </c>
       <c r="L7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" t="s">
         <v>25</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>29</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>7.9459999999999997</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>26</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>33</v>
       </c>
+      <c r="R7" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>46268</v>
       </c>
@@ -988,38 +1039,44 @@
       <c r="F8">
         <v>169309</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8">
+        <v>18624</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="3">
         <v>46311</v>
       </c>
-      <c r="I8" s="3">
+      <c r="J8" s="3">
         <v>46269</v>
       </c>
-      <c r="J8" t="s">
-        <v>24</v>
-      </c>
       <c r="K8" t="s">
         <v>24</v>
       </c>
       <c r="L8" t="s">
+        <v>24</v>
+      </c>
+      <c r="M8" t="s">
         <v>25</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>29</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>7.9459999999999997</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>26</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>33</v>
       </c>
+      <c r="R8" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>46268</v>
       </c>
@@ -1038,38 +1095,44 @@
       <c r="F9">
         <v>583451</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9">
+        <v>64180</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>46311</v>
       </c>
-      <c r="I9" s="3">
+      <c r="J9" s="3">
         <v>46269</v>
       </c>
-      <c r="J9" t="s">
-        <v>24</v>
-      </c>
       <c r="K9" t="s">
         <v>24</v>
       </c>
       <c r="L9" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" t="s">
         <v>25</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>29</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>7.9459999999999997</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>26</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>33</v>
       </c>
+      <c r="R9" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>46268</v>
       </c>
@@ -1088,38 +1151,44 @@
       <c r="F10">
         <v>19526146</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10">
+        <v>2147876</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>46311</v>
       </c>
-      <c r="I10" s="3">
+      <c r="J10" s="3">
         <v>46269</v>
       </c>
-      <c r="J10" t="s">
-        <v>24</v>
-      </c>
       <c r="K10" t="s">
         <v>24</v>
       </c>
       <c r="L10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" t="s">
         <v>25</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>29</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>52.673999999999999</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>26</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>36</v>
       </c>
+      <c r="R10" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>46268</v>
       </c>
@@ -1138,38 +1207,44 @@
       <c r="F11">
         <v>546601</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11">
+        <v>60126</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H11" s="3">
+      <c r="I11" s="3">
         <v>46311</v>
       </c>
-      <c r="I11" s="3">
+      <c r="J11" s="3">
         <v>46269</v>
       </c>
-      <c r="J11" t="s">
-        <v>24</v>
-      </c>
       <c r="K11" t="s">
         <v>24</v>
       </c>
       <c r="L11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M11" t="s">
         <v>25</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>29</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>52.673999999999999</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>26</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>36</v>
       </c>
+      <c r="R11" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>46268</v>
       </c>
@@ -1188,39 +1263,44 @@
       <c r="F12">
         <v>169309</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12">
+        <v>18624</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="3">
         <v>46311</v>
       </c>
-      <c r="I12" s="3">
+      <c r="J12" s="3">
         <v>46269</v>
       </c>
-      <c r="J12" t="s">
-        <v>24</v>
-      </c>
       <c r="K12" t="s">
         <v>24</v>
       </c>
       <c r="L12" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" t="s">
         <v>25</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>29</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>52.673999999999999</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>26</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>36</v>
       </c>
-      <c r="Q12" s="1"/>
+      <c r="R12" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>46268</v>
       </c>
@@ -1239,35 +1319,41 @@
       <c r="F13">
         <v>3867694</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13">
+        <v>425446</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="3">
+      <c r="I13" s="3">
         <v>46311</v>
       </c>
-      <c r="I13" s="3">
+      <c r="J13" s="3">
         <v>46269</v>
       </c>
-      <c r="J13" t="s">
-        <v>24</v>
-      </c>
       <c r="K13" t="s">
         <v>24</v>
       </c>
       <c r="L13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M13" t="s">
         <v>25</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>29</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>52.673999999999999</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>26</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>36</v>
+      </c>
+      <c r="R13" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>